<commit_message>
automation for all files in local folder
</commit_message>
<xml_diff>
--- a/examples/IOT-eDNA.xlsx
+++ b/examples/IOT-eDNA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau-my.sharepoint.com/personal/tak025_csiro_au/Documents/Documents/Miwa/IWY_eDNAdata/data_std/MS/submitted/supplementary/IOT-eDNA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24048977_student_uwa_edu_au/Documents/Documents/VS Code/FAIRe2MDT/FAIRe2MDT/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_4E4CCD934293EF5F88B3DABDC6C026963C6B129F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02E449F-448B-4E00-9404-93D99A6F7FA4}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_4E4CCD934293EF5F88B3DABDC6C026963C6B129F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7E7DF8B-F436-41E4-97CD-D6E041D36233}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2895" yWindow="1620" windowWidth="21600" windowHeight="11265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -10759,107 +10759,107 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.5">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.5">
+    <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="14.5">
+    <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="14.5">
+    <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="14.5">
+    <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.5">
+    <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="14.5">
+    <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.5">
+    <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.5">
+    <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="14.5">
+    <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="14.5">
+    <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="14.5">
+    <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.5">
+    <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.5">
+    <row r="14" spans="1:1">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.5">
+    <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="14.5">
+    <row r="16" spans="1:1">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="14.5">
+    <row r="17" spans="1:1">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.5">
+    <row r="18" spans="1:1">
       <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.5">
+    <row r="19" spans="1:1">
       <c r="A19" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.5">
+    <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
         <v>17</v>
       </c>
@@ -11913,12 +11913,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.5">
+    <row r="1" spans="1:6">
       <c r="A1" s="6" t="s">
         <v>32</v>
       </c>
@@ -11938,7 +11938,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.5">
+    <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
@@ -11952,7 +11952,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.5">
+    <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
         <v>42</v>
       </c>
@@ -11966,7 +11966,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="14.5">
+    <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
         <v>38</v>
       </c>
@@ -11980,7 +11980,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.5">
+    <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
@@ -11994,7 +11994,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="14.5">
+    <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
@@ -12008,7 +12008,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.5">
+    <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
         <v>42</v>
       </c>
@@ -12022,7 +12022,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.5">
+    <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
         <v>38</v>
       </c>
@@ -12036,7 +12036,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.5">
+    <row r="9" spans="1:6">
       <c r="A9" s="5" t="s">
         <v>55</v>
       </c>
@@ -12047,7 +12047,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.5">
+    <row r="10" spans="1:6">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -12061,7 +12061,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.5">
+    <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
         <v>38</v>
       </c>
@@ -12077,7 +12077,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" ht="14.5">
+    <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
         <v>61</v>
       </c>
@@ -12088,7 +12088,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.5">
+    <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
         <v>61</v>
       </c>
@@ -12102,7 +12102,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" ht="14.5">
+    <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
         <v>61</v>
       </c>
@@ -12116,7 +12116,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" ht="14.5">
+    <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
         <v>38</v>
       </c>
@@ -12130,7 +12130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.5">
+    <row r="16" spans="1:6">
       <c r="A16" s="4" t="s">
         <v>42</v>
       </c>
@@ -12141,7 +12141,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="14.5">
+    <row r="17" spans="1:6">
       <c r="A17" s="4" t="s">
         <v>42</v>
       </c>
@@ -12152,7 +12152,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.5">
+    <row r="18" spans="1:6">
       <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
@@ -12163,7 +12163,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="14.5">
+    <row r="19" spans="1:6">
       <c r="A19" s="4" t="s">
         <v>42</v>
       </c>
@@ -12174,7 +12174,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="14.5">
+    <row r="20" spans="1:6">
       <c r="A20" s="5" t="s">
         <v>55</v>
       </c>
@@ -14345,12 +14345,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:DZ274"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="130" width="11.453125" customWidth="1"/>
+    <col min="1" max="34" width="11.42578125" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="36" max="130" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:130" ht="14.5">
+    <row r="1" spans="1:130">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -14742,7 +14744,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:130" ht="14.5">
+    <row r="2" spans="1:130">
       <c r="A2" s="1" t="s">
         <v>206</v>
       </c>
@@ -15134,7 +15136,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="3" spans="1:130" ht="14.5">
+    <row r="3" spans="1:130">
       <c r="A3" s="6" t="s">
         <v>213</v>
       </c>
@@ -15526,7 +15528,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="4" spans="1:130" ht="14.5">
+    <row r="4" spans="1:130">
       <c r="A4" s="1" t="s">
         <v>342</v>
       </c>
@@ -15654,7 +15656,7 @@
       <c r="DX4" s="1"/>
       <c r="DZ4" s="1"/>
     </row>
-    <row r="5" spans="1:130" ht="14.5">
+    <row r="5" spans="1:130">
       <c r="A5" s="1" t="s">
         <v>356</v>
       </c>
@@ -15782,7 +15784,7 @@
       <c r="DX5" s="1"/>
       <c r="DZ5" s="1"/>
     </row>
-    <row r="6" spans="1:130" ht="14.5">
+    <row r="6" spans="1:130">
       <c r="A6" s="1" t="s">
         <v>358</v>
       </c>
@@ -15910,7 +15912,7 @@
       <c r="DX6" s="1"/>
       <c r="DZ6" s="1"/>
     </row>
-    <row r="7" spans="1:130" ht="14.5">
+    <row r="7" spans="1:130">
       <c r="A7" s="1" t="s">
         <v>360</v>
       </c>
@@ -16038,7 +16040,7 @@
       <c r="DX7" s="1"/>
       <c r="DZ7" s="1"/>
     </row>
-    <row r="8" spans="1:130" ht="14.5">
+    <row r="8" spans="1:130">
       <c r="A8" s="1" t="s">
         <v>362</v>
       </c>
@@ -16166,7 +16168,7 @@
       <c r="DX8" s="1"/>
       <c r="DZ8" s="1"/>
     </row>
-    <row r="9" spans="1:130" ht="14.5">
+    <row r="9" spans="1:130">
       <c r="A9" s="1" t="s">
         <v>364</v>
       </c>
@@ -16294,7 +16296,7 @@
       <c r="DX9" s="1"/>
       <c r="DZ9" s="1"/>
     </row>
-    <row r="10" spans="1:130" ht="14.5">
+    <row r="10" spans="1:130">
       <c r="A10" s="1" t="s">
         <v>366</v>
       </c>
@@ -16422,7 +16424,7 @@
       <c r="DX10" s="1"/>
       <c r="DZ10" s="1"/>
     </row>
-    <row r="11" spans="1:130" ht="14.5">
+    <row r="11" spans="1:130">
       <c r="A11" s="1" t="s">
         <v>368</v>
       </c>
@@ -16550,7 +16552,7 @@
       <c r="DX11" s="1"/>
       <c r="DZ11" s="1"/>
     </row>
-    <row r="12" spans="1:130" ht="14.5">
+    <row r="12" spans="1:130">
       <c r="A12" s="1" t="s">
         <v>370</v>
       </c>
@@ -16678,7 +16680,7 @@
       <c r="DX12" s="1"/>
       <c r="DZ12" s="1"/>
     </row>
-    <row r="13" spans="1:130" ht="14.5">
+    <row r="13" spans="1:130">
       <c r="A13" s="1" t="s">
         <v>372</v>
       </c>
@@ -16806,7 +16808,7 @@
       <c r="DX13" s="1"/>
       <c r="DZ13" s="1"/>
     </row>
-    <row r="14" spans="1:130" ht="14.5">
+    <row r="14" spans="1:130">
       <c r="A14" s="1" t="s">
         <v>374</v>
       </c>
@@ -16934,7 +16936,7 @@
       <c r="DX14" s="1"/>
       <c r="DZ14" s="1"/>
     </row>
-    <row r="15" spans="1:130" ht="14.5">
+    <row r="15" spans="1:130">
       <c r="A15" s="1" t="s">
         <v>376</v>
       </c>
@@ -17062,7 +17064,7 @@
       <c r="DX15" s="1"/>
       <c r="DZ15" s="1"/>
     </row>
-    <row r="16" spans="1:130" ht="14.5">
+    <row r="16" spans="1:130">
       <c r="A16" s="1" t="s">
         <v>378</v>
       </c>
@@ -17190,7 +17192,7 @@
       <c r="DX16" s="1"/>
       <c r="DZ16" s="1"/>
     </row>
-    <row r="17" spans="1:130" ht="14.5">
+    <row r="17" spans="1:130">
       <c r="A17" s="1" t="s">
         <v>380</v>
       </c>
@@ -17315,7 +17317,7 @@
       <c r="DX17" s="1"/>
       <c r="DZ17" s="1"/>
     </row>
-    <row r="18" spans="1:130" ht="14.5">
+    <row r="18" spans="1:130">
       <c r="A18" s="1" t="s">
         <v>382</v>
       </c>
@@ -17443,7 +17445,7 @@
       <c r="DX18" s="1"/>
       <c r="DZ18" s="1"/>
     </row>
-    <row r="19" spans="1:130" ht="14.5">
+    <row r="19" spans="1:130">
       <c r="A19" s="1" t="s">
         <v>384</v>
       </c>
@@ -17571,7 +17573,7 @@
       <c r="DX19" s="1"/>
       <c r="DZ19" s="1"/>
     </row>
-    <row r="20" spans="1:130" ht="14.5">
+    <row r="20" spans="1:130">
       <c r="A20" s="1" t="s">
         <v>386</v>
       </c>
@@ -45144,12 +45146,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:T1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="14.5">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -45211,7 +45213,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="14.5">
+    <row r="2" spans="1:20">
       <c r="A2" s="1" t="s">
         <v>206</v>
       </c>
@@ -45273,7 +45275,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="14.5">
+    <row r="3" spans="1:20">
       <c r="A3" s="6" t="s">
         <v>213</v>
       </c>
@@ -45335,7 +45337,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="14.5">
+    <row r="4" spans="1:20">
       <c r="A4" s="1" t="s">
         <v>342</v>
       </c>
@@ -45350,7 +45352,7 @@
       </c>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:20" ht="14.5">
+    <row r="5" spans="1:20">
       <c r="A5" s="1" t="s">
         <v>356</v>
       </c>
@@ -45365,7 +45367,7 @@
       </c>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:20" ht="14.5">
+    <row r="6" spans="1:20">
       <c r="A6" s="1" t="s">
         <v>358</v>
       </c>
@@ -45380,7 +45382,7 @@
       </c>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:20" ht="14.5">
+    <row r="7" spans="1:20">
       <c r="A7" s="1" t="s">
         <v>360</v>
       </c>
@@ -45395,7 +45397,7 @@
       </c>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="1:20" ht="14.5">
+    <row r="8" spans="1:20">
       <c r="A8" s="1" t="s">
         <v>362</v>
       </c>
@@ -45410,7 +45412,7 @@
       </c>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:20" ht="14.5">
+    <row r="9" spans="1:20">
       <c r="A9" s="1" t="s">
         <v>364</v>
       </c>
@@ -45425,7 +45427,7 @@
       </c>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:20" ht="14.5">
+    <row r="10" spans="1:20">
       <c r="A10" s="1" t="s">
         <v>366</v>
       </c>
@@ -45440,7 +45442,7 @@
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:20" ht="14.5">
+    <row r="11" spans="1:20">
       <c r="A11" s="1" t="s">
         <v>368</v>
       </c>
@@ -45455,7 +45457,7 @@
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:20" ht="14.5">
+    <row r="12" spans="1:20">
       <c r="A12" s="1" t="s">
         <v>370</v>
       </c>
@@ -45470,7 +45472,7 @@
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:20" ht="14.5">
+    <row r="13" spans="1:20">
       <c r="A13" s="1" t="s">
         <v>372</v>
       </c>
@@ -45485,7 +45487,7 @@
       </c>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:20" ht="14.5">
+    <row r="14" spans="1:20">
       <c r="A14" s="1" t="s">
         <v>374</v>
       </c>
@@ -45500,7 +45502,7 @@
       </c>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:20" ht="14.5">
+    <row r="15" spans="1:20">
       <c r="A15" s="1" t="s">
         <v>376</v>
       </c>
@@ -45515,7 +45517,7 @@
       </c>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:20" ht="14.5">
+    <row r="16" spans="1:20">
       <c r="A16" s="1" t="s">
         <v>378</v>
       </c>
@@ -45530,7 +45532,7 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" ht="14.5">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
         <v>380</v>
       </c>
@@ -45545,7 +45547,7 @@
       </c>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" ht="14.5">
+    <row r="18" spans="1:7">
       <c r="A18" s="1" t="s">
         <v>382</v>
       </c>
@@ -45560,7 +45562,7 @@
       </c>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" ht="14.5">
+    <row r="19" spans="1:7">
       <c r="A19" s="1" t="s">
         <v>384</v>
       </c>
@@ -45575,7 +45577,7 @@
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" ht="14.5">
+    <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
         <v>386</v>
       </c>
@@ -53500,12 +53502,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:U1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="14.5">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -53570,7 +53572,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="14.5">
+    <row r="2" spans="1:21">
       <c r="A2" s="1" t="s">
         <v>206</v>
       </c>
@@ -53635,7 +53637,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="14.5">
+    <row r="3" spans="1:21">
       <c r="A3" s="6" t="s">
         <v>1188</v>
       </c>
@@ -53700,55 +53702,55 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="14.5">
+    <row r="4" spans="1:21">
       <c r="L4" s="1"/>
     </row>
-    <row r="5" spans="1:21" ht="14.5">
+    <row r="5" spans="1:21">
       <c r="L5" s="1"/>
     </row>
-    <row r="6" spans="1:21" ht="14.5">
+    <row r="6" spans="1:21">
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:21" ht="14.5">
+    <row r="7" spans="1:21">
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:21" ht="14.5">
+    <row r="8" spans="1:21">
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="1:21" ht="14.5">
+    <row r="9" spans="1:21">
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:21" ht="14.5">
+    <row r="10" spans="1:21">
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:21" ht="14.5">
+    <row r="11" spans="1:21">
       <c r="L11" s="1"/>
     </row>
-    <row r="12" spans="1:21" ht="14.5">
+    <row r="12" spans="1:21">
       <c r="L12" s="1"/>
     </row>
-    <row r="13" spans="1:21" ht="14.5">
+    <row r="13" spans="1:21">
       <c r="L13" s="1"/>
     </row>
-    <row r="14" spans="1:21" ht="14.5">
+    <row r="14" spans="1:21">
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:21" ht="14.5">
+    <row r="15" spans="1:21">
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:21" ht="14.5">
+    <row r="16" spans="1:21">
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="12:12" ht="14.5">
+    <row r="17" spans="12:12">
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="12:12" ht="14.5">
+    <row r="18" spans="12:12">
       <c r="L18" s="1"/>
     </row>
-    <row r="19" spans="12:12" ht="14.5">
+    <row r="19" spans="12:12">
       <c r="L19" s="1"/>
     </row>
-    <row r="20" spans="12:12" ht="14.5">
+    <row r="20" spans="12:12">
       <c r="L20" s="1"/>
     </row>
     <row r="21" spans="12:12" ht="15.75" customHeight="1">
@@ -54919,12 +54921,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:U1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="14.5">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -54989,7 +54991,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="14.5">
+    <row r="2" spans="1:21">
       <c r="A2" s="1" t="s">
         <v>206</v>
       </c>
@@ -55054,7 +55056,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="14.5">
+    <row r="3" spans="1:21">
       <c r="A3" s="6" t="s">
         <v>1188</v>
       </c>
@@ -55119,55 +55121,55 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="14.5">
+    <row r="4" spans="1:21">
       <c r="L4" s="1"/>
     </row>
-    <row r="5" spans="1:21" ht="14.5">
+    <row r="5" spans="1:21">
       <c r="L5" s="1"/>
     </row>
-    <row r="6" spans="1:21" ht="14.5">
+    <row r="6" spans="1:21">
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:21" ht="14.5">
+    <row r="7" spans="1:21">
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:21" ht="14.5">
+    <row r="8" spans="1:21">
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="1:21" ht="14.5">
+    <row r="9" spans="1:21">
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:21" ht="14.5">
+    <row r="10" spans="1:21">
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:21" ht="14.5">
+    <row r="11" spans="1:21">
       <c r="L11" s="1"/>
     </row>
-    <row r="12" spans="1:21" ht="14.5">
+    <row r="12" spans="1:21">
       <c r="L12" s="1"/>
     </row>
-    <row r="13" spans="1:21" ht="14.5">
+    <row r="13" spans="1:21">
       <c r="L13" s="1"/>
     </row>
-    <row r="14" spans="1:21" ht="14.5">
+    <row r="14" spans="1:21">
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:21" ht="14.5">
+    <row r="15" spans="1:21">
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:21" ht="14.5">
+    <row r="16" spans="1:21">
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="12:12" ht="14.5">
+    <row r="17" spans="12:12">
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="12:12" ht="14.5">
+    <row r="18" spans="12:12">
       <c r="L18" s="1"/>
     </row>
-    <row r="19" spans="12:12" ht="14.5">
+    <row r="19" spans="12:12">
       <c r="L19" s="1"/>
     </row>
-    <row r="20" spans="12:12" ht="14.5">
+    <row r="20" spans="12:12">
       <c r="L20" s="1"/>
     </row>
     <row r="21" spans="12:12" ht="15.75" customHeight="1">
@@ -56338,12 +56340,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AF1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="32" width="11.453125" customWidth="1"/>
+    <col min="1" max="32" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="14.5">
+    <row r="1" spans="1:32">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -56441,7 +56443,7 @@
         <v>1239</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="14.5">
+    <row r="2" spans="1:32">
       <c r="A2" s="1" t="s">
         <v>59</v>
       </c>
@@ -56464,7 +56466,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="3" spans="1:32" ht="14.5">
+    <row r="3" spans="1:32">
       <c r="A3" s="1" t="s">
         <v>63</v>
       </c>
@@ -56484,7 +56486,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="4" spans="1:32" ht="14.5">
+    <row r="4" spans="1:32">
       <c r="A4" s="1" t="s">
         <v>64</v>
       </c>
@@ -56504,7 +56506,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="5" spans="1:32" ht="14.5">
+    <row r="5" spans="1:32">
       <c r="A5" s="1" t="s">
         <v>214</v>
       </c>
@@ -56533,7 +56535,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="14.5">
+    <row r="6" spans="1:32">
       <c r="A6" s="1" t="s">
         <v>215</v>
       </c>
@@ -56565,7 +56567,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="14.5">
+    <row r="7" spans="1:32">
       <c r="A7" s="1" t="s">
         <v>225</v>
       </c>
@@ -56591,7 +56593,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="14.5">
+    <row r="8" spans="1:32">
       <c r="A8" s="1" t="s">
         <v>226</v>
       </c>
@@ -56629,7 +56631,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="14.5">
+    <row r="9" spans="1:32">
       <c r="A9" s="1" t="s">
         <v>235</v>
       </c>
@@ -56649,7 +56651,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="14.5">
+    <row r="10" spans="1:32">
       <c r="A10" s="1" t="s">
         <v>239</v>
       </c>
@@ -56693,7 +56695,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="14.5">
+    <row r="11" spans="1:32">
       <c r="A11" s="1" t="s">
         <v>241</v>
       </c>
@@ -56725,7 +56727,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="14.5">
+    <row r="12" spans="1:32">
       <c r="A12" s="1" t="s">
         <v>247</v>
       </c>
@@ -56745,7 +56747,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="14.5">
+    <row r="13" spans="1:32">
       <c r="A13" s="1" t="s">
         <v>250</v>
       </c>
@@ -56780,7 +56782,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="14.5">
+    <row r="14" spans="1:32">
       <c r="A14" s="1" t="s">
         <v>256</v>
       </c>
@@ -56818,7 +56820,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="14.5">
+    <row r="15" spans="1:32">
       <c r="A15" s="1" t="s">
         <v>258</v>
       </c>
@@ -56844,7 +56846,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="14.5">
+    <row r="16" spans="1:32">
       <c r="A16" s="1" t="s">
         <v>263</v>
       </c>
@@ -56876,7 +56878,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="17" spans="1:32" ht="14.5">
+    <row r="17" spans="1:32">
       <c r="A17" s="1" t="s">
         <v>268</v>
       </c>
@@ -56920,7 +56922,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="18" spans="1:32" ht="14.5">
+    <row r="18" spans="1:32">
       <c r="A18" s="1" t="s">
         <v>269</v>
       </c>
@@ -56952,7 +56954,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="19" spans="1:32" ht="14.5">
+    <row r="19" spans="1:32">
       <c r="A19" s="1" t="s">
         <v>270</v>
       </c>
@@ -56987,7 +56989,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="20" spans="1:32" ht="14.5">
+    <row r="20" spans="1:32">
       <c r="A20" s="1" t="s">
         <v>274</v>
       </c>

</xml_diff>